<commit_message>
feat(mpr,reports,mtrix,ecom): análisis trazabilidad, filtros PV y mejoras varias
Análisis trazabilidad canónico (kardex): Stock Inicial, columna Conteo, KPIs demanda,
reconstrucción de saldo y UI por nombre de artículo. Reportes filtros PV/sucursal,
mtrix proveedores/export, ecom pedido masivo y documentación de auditoría.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/reports/templates/reports/excel/monthly_reporting/levis_bw_annual.xlsx
+++ b/reports/templates/reports/excel/monthly_reporting/levis_bw_annual.xlsx
@@ -55,7 +55,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,9 +421,115 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:F4"/>
+  <dimension ref="A2:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="2">
+      <c r="E2">
+        <f>SUM(E5:E4931)</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>SUM(F5:F4931)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUM(G5:G4931)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUM(H5:H4931)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUM(I5:I4931)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUM(J5:J4931)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUM(K5:K4931)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUM(L5:L4931)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUM(M5:M4931)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUM(N5:N4931)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUM(O5:O4931)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>SUM(P5:P4931)</f>
+        <v/>
+      </c>
+      <c r="Q2">
+        <f>SUM(Q5:Q4931)</f>
+        <v/>
+      </c>
+      <c r="R2">
+        <f>SUM(R5:R4931)</f>
+        <v/>
+      </c>
+      <c r="S2">
+        <f>SUM(S5:S4931)</f>
+        <v/>
+      </c>
+      <c r="T2">
+        <f>SUM(T5:T4931)</f>
+        <v/>
+      </c>
+      <c r="U2">
+        <f>SUM(U5:U4931)</f>
+        <v/>
+      </c>
+      <c r="V2">
+        <f>SUM(V5:V4931)</f>
+        <v/>
+      </c>
+      <c r="W2">
+        <f>SUM(W5:W4931)</f>
+        <v/>
+      </c>
+      <c r="X2">
+        <f>SUM(X5:X4931)</f>
+        <v/>
+      </c>
+      <c r="Y2">
+        <f>SUM(Y5:Y4931)</f>
+        <v/>
+      </c>
+      <c r="Z2">
+        <f>SUM(Z5:Z4931)</f>
+        <v/>
+      </c>
+      <c r="AA2">
+        <f>SUM(AA5:AA4931)</f>
+        <v/>
+      </c>
+      <c r="AB2">
+        <f>SUM(AB5:AB4931)</f>
+        <v/>
+      </c>
+      <c r="AC2">
+        <f>SUM(AC5:AC4931)</f>
+        <v/>
+      </c>
+      <c r="AD2">
+        <f>SUM(AD5:AD4931)</f>
+        <v/>
+      </c>
+    </row>
     <row r="3">
       <c r="E3" t="inlineStr">
         <is>
@@ -431,6 +537,116 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>amounts</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>amounts</t>
         </is>
@@ -444,7 +660,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>City / Province</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -459,6 +675,49 @@
       </c>
       <c r="E4" s="2" t="n">
         <v>46023</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>46054</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>46143</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="Y4" s="2" t="n">
+        <v>46327</v>
+      </c>
+      <c r="AA4" s="2" t="n">
+        <v>46357</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>YTD_Units</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>YTD_Sales</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>